<commit_message>
Update internship timesheet for Day 4
</commit_message>
<xml_diff>
--- a/timesheet/Dhanu.xlsx
+++ b/timesheet/Dhanu.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
   <si>
     <t>Date</t>
   </si>
@@ -113,7 +113,26 @@
     <t>Focus on business formulas and create KPI sheet for sample sales dataset(Maven Coffee Shop dataset)</t>
   </si>
   <si>
+    <t>https://github.com/dhanusree-prof/mvj-internship-data-analytics/commit/5bf67cb8e67b7237e9de11f9f9dac68e03f9d908</t>
+  </si>
+  <si>
     <t xml:space="preserve">yes - to learn the formulas </t>
+  </si>
+  <si>
+    <t>24.10.2026</t>
+  </si>
+  <si>
+    <t>Build a what-if model: 'what price and footfall hit a revenue target?' and Start Project 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/dhanusree-prof/mvj-internship-data-analytics/commit/541ae09cc81f54ef91d0646bdc7a1b3d3cec7f55
+</t>
+  </si>
+  <si>
+    <t>yes - excel online didnt have forecast sheet features to do what-if analysis, so checked how it can be done manually</t>
+  </si>
+  <si>
+    <t>learned to use formula based alternative since forecast feature was unavailable</t>
   </si>
 </sst>
 </file>
@@ -1275,7 +1294,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.2727272727273" customWidth="1"/>
@@ -1423,24 +1442,53 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" ht="29" spans="1:10">
+    <row r="10" ht="58" spans="1:10">
       <c r="A10" t="s">
         <v>17</v>
       </c>
       <c r="B10">
         <v>7</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>27</v>
       </c>
       <c r="G10" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="H10" s="2" t="s">
         <v>28</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="J10" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="11" ht="87" spans="1:11">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11">
+        <v>8</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J11" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete day 5 SQL aggregation analysis
</commit_message>
<xml_diff>
--- a/timesheet/Dhanu.xlsx
+++ b/timesheet/Dhanu.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
   <si>
     <t>Date</t>
   </si>
@@ -133,6 +133,18 @@
   </si>
   <si>
     <t>learned to use formula based alternative since forecast feature was unavailable</t>
+  </si>
+  <si>
+    <t>25.10.2026</t>
+  </si>
+  <si>
+    <t>Load Online Retail II into SQLite or DuckDB and calculate Revenue, orders, average order value by month and country. Documented preliminary findings and calculation limitations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes - for writing SQL aggregation queries for monthly and country-level revenue, order counts, and average order value. </t>
+  </si>
+  <si>
+    <t>SQL aggregation queries</t>
   </si>
 </sst>
 </file>
@@ -1294,7 +1306,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.2727272727273" customWidth="1"/>
@@ -1478,7 +1490,7 @@
       <c r="G11" t="s">
         <v>19</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H11" s="2" t="s">
         <v>32</v>
       </c>
       <c r="I11" s="2" t="s">
@@ -1489,6 +1501,29 @@
       </c>
       <c r="K11" s="2" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="12" ht="87" spans="1:11">
+      <c r="A12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12">
+        <v>9</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G12" t="s">
+        <v>19</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="J12" t="s">
+        <v>22</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Day 06: add customer analysis with SQL joins and segments
</commit_message>
<xml_diff>
--- a/timesheet/Dhanu.xlsx
+++ b/timesheet/Dhanu.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
   <si>
     <t>Date</t>
   </si>
@@ -139,6 +139,9 @@
   </si>
   <si>
     <t>Load Online Retail II into SQLite or DuckDB and calculate Revenue, orders, average order value by month and country. Documented preliminary findings and calculation limitations.</t>
+  </si>
+  <si>
+    <t>https://github.com/dhanusree-prof/mvj-internship-data-analytics/commit/e52c647d324cbf618750fe9a850e82b99ed74fdd</t>
   </si>
   <si>
     <t xml:space="preserve">yes - for writing SQL aggregation queries for monthly and country-level revenue, order counts, and average order value. </t>
@@ -1510,20 +1513,23 @@
       <c r="B12">
         <v>9</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>36</v>
       </c>
       <c r="G12" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="H12" s="3" t="s">
         <v>37</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="J12" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="3" t="s">
-        <v>38</v>
+      <c r="K12" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Day 06: updated timesheet with commit link
</commit_message>
<xml_diff>
--- a/timesheet/Dhanu.xlsx
+++ b/timesheet/Dhanu.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="45">
   <si>
     <t>Date</t>
   </si>
@@ -148,6 +148,24 @@
   </si>
   <si>
     <t>SQL aggregation queries</t>
+  </si>
+  <si>
+    <t>26.10.206</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Creating 
+Customer-level table with joins and CASE-based segments.</t>
+  </si>
+  <si>
+    <t>https://github.com/dhanusree-prof/mvj-internship-data-analytics/commit/a78cc9c8c592826d521c80f7d676159eeb606061</t>
+  </si>
+  <si>
+    <t>yes -  for the explanation of
+ SQL structure, help develop queries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">usage of joins and CASE
+</t>
   </si>
 </sst>
 </file>
@@ -1309,7 +1327,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.2727272727273" customWidth="1"/>
@@ -1519,7 +1537,7 @@
       <c r="G12" t="s">
         <v>19</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="2" t="s">
         <v>37</v>
       </c>
       <c r="I12" s="2" t="s">
@@ -1530,6 +1548,32 @@
       </c>
       <c r="K12" s="2" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="13" ht="58" spans="1:11">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13">
+        <v>10</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G13" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="J13" t="s">
+        <v>22</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Day 7: analyse retail trends with SQL window functions
</commit_message>
<xml_diff>
--- a/timesheet/Dhanu.xlsx
+++ b/timesheet/Dhanu.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
   <si>
     <t>Date</t>
   </si>
@@ -166,6 +166,18 @@
   <si>
     <t xml:space="preserve">usage of joins and CASE
 </t>
+  </si>
+  <si>
+    <t>27.10.2026</t>
+  </si>
+  <si>
+    <t>Preparing monthly sales, calculating running totals and month-on-month growth with LAG, ranked products by country, and analysed first-purchase cohorts.</t>
+  </si>
+  <si>
+    <t>yes - for SQL validation</t>
+  </si>
+  <si>
+    <t>Practised SQL window functions</t>
   </si>
 </sst>
 </file>
@@ -1327,7 +1339,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.2727272727273" customWidth="1"/>
@@ -1557,23 +1569,46 @@
       <c r="B13">
         <v>10</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="2" t="s">
         <v>41</v>
       </c>
       <c r="G13" t="s">
         <v>19</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="I13" s="2" t="s">
         <v>43</v>
       </c>
       <c r="J13" t="s">
         <v>22</v>
       </c>
-      <c r="K13" s="3" t="s">
+      <c r="K13" s="2" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="14" ht="58" spans="1:11">
+      <c r="A14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14">
+        <v>11</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" t="s">
+        <v>47</v>
+      </c>
+      <c r="J14" t="s">
+        <v>22</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Day 7 timesheet updated with commit link
</commit_message>
<xml_diff>
--- a/timesheet/Dhanu.xlsx
+++ b/timesheet/Dhanu.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="50">
   <si>
     <t>Date</t>
   </si>
@@ -172,6 +172,9 @@
   </si>
   <si>
     <t>Preparing monthly sales, calculating running totals and month-on-month growth with LAG, ranked products by country, and analysed first-purchase cohorts.</t>
+  </si>
+  <si>
+    <t>https://github.com/dhanusree-prof/mvj-internship-data-analytics/commit/d67c877c6418d22d9ac6550bbaa35ce550e15fa6</t>
   </si>
   <si>
     <t>yes - for SQL validation</t>
@@ -1601,14 +1604,17 @@
       <c r="G14" t="s">
         <v>19</v>
       </c>
+      <c r="H14" s="3" t="s">
+        <v>47</v>
+      </c>
       <c r="I14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J14" t="s">
         <v>22</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated day 08 timesheet
</commit_message>
<xml_diff>
--- a/timesheet/Dhanu.xlsx
+++ b/timesheet/Dhanu.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="54">
   <si>
     <t>Date</t>
   </si>
@@ -181,6 +181,18 @@
   </si>
   <si>
     <t>Practised SQL window functions</t>
+  </si>
+  <si>
+    <t>Completed Project 1 KPI analysis using SQL and Excel on the Online Retail II dataset. Calculated net sales proxy, orders, AOV, repeat customer rate, top products, and monthly growth. Prepared the Excel KPI pack and five evidence-based recommendations</t>
+  </si>
+  <si>
+    <t>https://github.com/dhanusree-prof/mvj-internship-data-analytics/commit/db54a5eb08e9c7c92deb2bceea4f9c021d43627a</t>
+  </si>
+  <si>
+    <t>yes - for cross checking the results obtained after analysis</t>
+  </si>
+  <si>
+    <t>To do KPI analysis using SQL and Excel</t>
   </si>
 </sst>
 </file>
@@ -1342,7 +1354,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.2727272727273" customWidth="1"/>
@@ -1598,13 +1610,13 @@
       <c r="B14">
         <v>11</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="2" t="s">
         <v>46</v>
       </c>
       <c r="G14" t="s">
         <v>19</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="H14" s="2" t="s">
         <v>47</v>
       </c>
       <c r="I14" t="s">
@@ -1613,8 +1625,34 @@
       <c r="J14" t="s">
         <v>22</v>
       </c>
-      <c r="K14" s="3" t="s">
+      <c r="K14" s="2" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="15" ht="72.5" spans="1:11">
+      <c r="A15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15">
+        <v>11</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" t="s">
+        <v>19</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J15" t="s">
+        <v>22</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>